<commit_message>
atualizacao com os requisitos
</commit_message>
<xml_diff>
--- a/data/cepea-consulta-açucar-santos.reparado.xlsx
+++ b/data/cepea-consulta-açucar-santos.reparado.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filipe.guidastri\Documents\Projetos\painel-controle-commodities\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\filipe.guidastri\Documents\Projetos\acompanhamento-cotacao\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{745EDFB7-299C-49E2-8DE1-A1EEFF10BE76}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9A447FE1-CF56-4151-8089-2482A261CB09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5760" yWindow="3396" windowWidth="17280" windowHeight="8964"/>
   </bookViews>

</xml_diff>